<commit_message>
docs: quita las últimas menciones al despliegue anterior
</commit_message>
<xml_diff>
--- a/docs/qa/Plan_de_pruebas_Sprint_1-3.xlsx
+++ b/docs/qa/Plan_de_pruebas_Sprint_1-3.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Parte A - Manuales'!$A$1:$M$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pasos TC'!$A$1:$E$90</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Parte B - Automatizados'!$A$1:$L$431</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defectos y pendientes'!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Defectos y pendientes'!$A$1:$F$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -38813,7 +38813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -39167,12 +39167,12 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>VPS de Dokku: SSH (puerto 22) y HTTP no responden, por lo que no se pudo borrar la aplicación ni sus datos en el servidor.</t>
+          <t>Las ramas dev-backend y dev-frontend no tienen los cambios de dev.</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Infraestructura</t>
+          <t>Git</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -39182,7 +39182,7 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>En el repositorio se eliminaron el Dockerfile y el nginx.conf de producción del frontend y las referencias en la documentación.</t>
+          <t>Sincronizar por PR antes de que sigan Emir y Belén.</t>
         </is>
       </c>
     </row>
@@ -39197,12 +39197,12 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Las ramas dev-backend y dev-frontend no tienen los cambios de dev.</t>
+          <t>Jira: SCRUM-198 y SCRUM-215 (QA) siguen 'En curso'.</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Git</t>
+          <t>Jira</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -39212,42 +39212,12 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Sincronizar por PR antes de que sigan Emir y Belén.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>Jira: SCRUM-198 y SCRUM-215 (QA) siguen 'En curso'.</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Jira</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Abierta</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
           <t>Cerrar con el resultado de esta ejecución.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14"/>
+  <autoFilter ref="A1:F13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>